<commit_message>
LoginAPI excel data provider and ran test with same
</commit_message>
<xml_diff>
--- a/src/test/resources/testData/PhoenixTestData.xlsx
+++ b/src/test/resources/testData/PhoenixTestData.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="3">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="5">
   <si>
     <t>username</t>
   </si>
@@ -21,6 +21,12 @@
   </si>
   <si>
     <t>iamfd</t>
+  </si>
+  <si>
+    <t>iamsup</t>
+  </si>
+  <si>
+    <t>iameng</t>
   </si>
 </sst>
 </file>
@@ -298,6 +304,22 @@
         <v>1</v>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>1</v>
+      </c>
+    </row>
   </sheetData>
   <drawing r:id="rId1"/>
 </worksheet>

</xml_diff>

<commit_message>
ExcelUtil enhanced to support CreateJob API
</commit_message>
<xml_diff>
--- a/src/test/resources/testData/PhoenixTestData.xlsx
+++ b/src/test/resources/testData/PhoenixTestData.xlsx
@@ -4,7 +4,7 @@
   <workbookPr/>
   <sheets>
     <sheet state="visible" name="LoginTestData" sheetId="1" r:id="rId5"/>
-    <sheet state="visible" name="Sheet2" sheetId="2" r:id="rId6"/>
+    <sheet state="visible" name="CreateJobTestData" sheetId="2" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr/>
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="5">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="105" uniqueCount="51">
   <si>
     <t>username</t>
   </si>
@@ -27,13 +27,151 @@
   </si>
   <si>
     <t>iameng</t>
+  </si>
+  <si>
+    <t>mst_service_location_id</t>
+  </si>
+  <si>
+    <t>mst_platform_id</t>
+  </si>
+  <si>
+    <t>mst_warrenty_status_id</t>
+  </si>
+  <si>
+    <t>mst_oem_id</t>
+  </si>
+  <si>
+    <t>customer__first_name</t>
+  </si>
+  <si>
+    <t>customer__last_name</t>
+  </si>
+  <si>
+    <t>customer__mobile_number</t>
+  </si>
+  <si>
+    <t>customer__mobile_number_alt</t>
+  </si>
+  <si>
+    <t>customer__email_id</t>
+  </si>
+  <si>
+    <t>customer__email_id_alt</t>
+  </si>
+  <si>
+    <t>customer_address__flat_number</t>
+  </si>
+  <si>
+    <t>customer_address__apartment_name</t>
+  </si>
+  <si>
+    <t>customer_address__street_name</t>
+  </si>
+  <si>
+    <t>customer_address__landmark</t>
+  </si>
+  <si>
+    <t>customer_address__area</t>
+  </si>
+  <si>
+    <t>customer_address__pincode</t>
+  </si>
+  <si>
+    <t>customer_address__country</t>
+  </si>
+  <si>
+    <t>customer_address__state</t>
+  </si>
+  <si>
+    <t>customer_product__dop</t>
+  </si>
+  <si>
+    <t>customer_product__serial_number</t>
+  </si>
+  <si>
+    <t>customer_product__imei1</t>
+  </si>
+  <si>
+    <t>customer_product__imei2</t>
+  </si>
+  <si>
+    <t>customer_product__popurl</t>
+  </si>
+  <si>
+    <t>customer_product__product_id</t>
+  </si>
+  <si>
+    <t>customer_product__mst_model_id</t>
+  </si>
+  <si>
+    <t>problems__id</t>
+  </si>
+  <si>
+    <t>problems__remark</t>
+  </si>
+  <si>
+    <t>Tamia</t>
+  </si>
+  <si>
+    <t>McLaughlin</t>
+  </si>
+  <si>
+    <t>799-639-2770</t>
+  </si>
+  <si>
+    <t>Vincent_Rippin@yahoo.com</t>
+  </si>
+  <si>
+    <t>c 304</t>
+  </si>
+  <si>
+    <t>Jupiter</t>
+  </si>
+  <si>
+    <t>MG road</t>
+  </si>
+  <si>
+    <t>Bangur Nagar</t>
+  </si>
+  <si>
+    <t>Goregaon West</t>
+  </si>
+  <si>
+    <t>India</t>
+  </si>
+  <si>
+    <t>Maharashtra</t>
+  </si>
+  <si>
+    <t>2025-04-06T18:30:00.000Z</t>
+  </si>
+  <si>
+    <t>Battery Issue</t>
+  </si>
+  <si>
+    <t>Jack</t>
+  </si>
+  <si>
+    <t>Nive</t>
+  </si>
+  <si>
+    <t>MS</t>
+  </si>
+  <si>
+    <t>Dhoni</t>
+  </si>
+  <si>
+    <t>Ruturaj</t>
+  </si>
+  <si>
+    <t>Gaikwad</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <fonts count="2">
+  <fonts count="4">
     <font>
       <sz val="10.0"/>
       <color rgb="FF000000"/>
@@ -45,13 +183,29 @@
       <name val="Arial"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11.0"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="9.0"/>
+      <color rgb="FF2A00FF"/>
+      <name val="Arial"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="lightGray"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFFF"/>
+        <bgColor rgb="FFFFFFFF"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -60,11 +214,20 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="5">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="right" readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
+    </xf>
+    <xf borderId="0" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
   </cellXfs>
@@ -331,7 +494,501 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
   <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
-  <sheetData/>
+  <cols>
+    <col customWidth="1" min="1" max="1" width="19.13"/>
+    <col customWidth="1" min="2" max="2" width="13.38"/>
+    <col customWidth="1" min="3" max="3" width="19.0"/>
+    <col customWidth="1" min="4" max="4" width="10.38"/>
+    <col customWidth="1" min="6" max="6" width="17.63"/>
+    <col customWidth="1" min="7" max="7" width="21.75"/>
+    <col customWidth="1" min="8" max="8" width="24.63"/>
+    <col customWidth="1" min="19" max="19" width="21.13"/>
+    <col customWidth="1" min="20" max="20" width="27.38"/>
+    <col customWidth="1" min="21" max="22" width="20.75"/>
+    <col customWidth="1" min="23" max="23" width="21.5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="I1" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="J1" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="K1" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="L1" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="M1" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="N1" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="O1" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="P1" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="Q1" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="R1" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="S1" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="T1" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="U1" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="V1" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="W1" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="X1" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y1" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="Z1" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="AA1" s="2" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="3">
+        <v>0.0</v>
+      </c>
+      <c r="B2" s="3">
+        <v>2.0</v>
+      </c>
+      <c r="C2" s="3">
+        <v>1.0</v>
+      </c>
+      <c r="D2" s="3">
+        <v>1.0</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="G2" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="I2" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="K2" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="L2" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="M2" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="N2" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="O2" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="P2" s="3">
+        <v>411039.0</v>
+      </c>
+      <c r="Q2" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="R2" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="S2" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="T2" s="4">
+        <v>1.9181303511419E13</v>
+      </c>
+      <c r="U2" s="4">
+        <v>1.9181303511419E13</v>
+      </c>
+      <c r="V2" s="4">
+        <v>1.9181303511419E13</v>
+      </c>
+      <c r="W2" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="X2" s="3">
+        <v>1.0</v>
+      </c>
+      <c r="Y2" s="3">
+        <v>1.0</v>
+      </c>
+      <c r="Z2" s="3">
+        <v>1.0</v>
+      </c>
+      <c r="AA2" s="2" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3">
+        <v>0.0</v>
+      </c>
+      <c r="B3" s="3">
+        <v>2.0</v>
+      </c>
+      <c r="C3" s="3">
+        <v>1.0</v>
+      </c>
+      <c r="D3" s="3">
+        <v>1.0</v>
+      </c>
+      <c r="E3" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="F3" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="G3" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="I3" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="K3" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="L3" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="M3" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="N3" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="O3" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="P3" s="3">
+        <v>411039.0</v>
+      </c>
+      <c r="Q3" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="R3" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="S3" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="T3" s="4">
+        <v>1.918130351142E13</v>
+      </c>
+      <c r="U3" s="4">
+        <v>1.918130351142E13</v>
+      </c>
+      <c r="V3" s="4">
+        <v>1.918130351142E13</v>
+      </c>
+      <c r="W3" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="X3" s="3">
+        <v>1.0</v>
+      </c>
+      <c r="Y3" s="3">
+        <v>1.0</v>
+      </c>
+      <c r="Z3" s="3">
+        <v>1.0</v>
+      </c>
+      <c r="AA3" s="2" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3">
+        <v>0.0</v>
+      </c>
+      <c r="B4" s="3">
+        <v>2.0</v>
+      </c>
+      <c r="C4" s="3">
+        <v>1.0</v>
+      </c>
+      <c r="D4" s="3">
+        <v>1.0</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="F4" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="G4" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="I4" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="K4" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="L4" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="M4" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="N4" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="O4" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="P4" s="3">
+        <v>411039.0</v>
+      </c>
+      <c r="Q4" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="R4" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="S4" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="T4" s="4">
+        <v>1.9181303511421E13</v>
+      </c>
+      <c r="U4" s="4">
+        <v>1.9181303511421E13</v>
+      </c>
+      <c r="V4" s="4">
+        <v>1.9181303511421E13</v>
+      </c>
+      <c r="W4" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="X4" s="3">
+        <v>1.0</v>
+      </c>
+      <c r="Y4" s="3">
+        <v>1.0</v>
+      </c>
+      <c r="Z4" s="3">
+        <v>1.0</v>
+      </c>
+      <c r="AA4" s="2" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3">
+        <v>0.0</v>
+      </c>
+      <c r="B5" s="3">
+        <v>2.0</v>
+      </c>
+      <c r="C5" s="3">
+        <v>1.0</v>
+      </c>
+      <c r="D5" s="3">
+        <v>1.0</v>
+      </c>
+      <c r="E5" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="F5" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="G5" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="I5" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="K5" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="L5" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="M5" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="N5" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="O5" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="P5" s="3">
+        <v>411039.0</v>
+      </c>
+      <c r="Q5" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="R5" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="S5" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="T5" s="4">
+        <v>1.9181303511422E13</v>
+      </c>
+      <c r="U5" s="4">
+        <v>1.9181303511422E13</v>
+      </c>
+      <c r="V5" s="4">
+        <v>1.9181303511422E13</v>
+      </c>
+      <c r="W5" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="X5" s="3">
+        <v>1.0</v>
+      </c>
+      <c r="Y5" s="3">
+        <v>1.0</v>
+      </c>
+      <c r="Z5" s="3">
+        <v>1.0</v>
+      </c>
+      <c r="AA5" s="2" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3">
+        <v>0.0</v>
+      </c>
+      <c r="B6" s="3">
+        <v>2.0</v>
+      </c>
+      <c r="C6" s="3">
+        <v>1.0</v>
+      </c>
+      <c r="D6" s="3">
+        <v>1.0</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="F6" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="G6" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="I6" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="K6" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="L6" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="M6" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="N6" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="O6" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="P6" s="3">
+        <v>411039.0</v>
+      </c>
+      <c r="Q6" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="R6" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="S6" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="T6" s="4">
+        <v>1.9181303511423E13</v>
+      </c>
+      <c r="U6" s="4">
+        <v>1.9181303511423E13</v>
+      </c>
+      <c r="V6" s="4">
+        <v>1.9181303511423E13</v>
+      </c>
+      <c r="W6" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="X6" s="3">
+        <v>1.0</v>
+      </c>
+      <c r="Y6" s="3">
+        <v>1.0</v>
+      </c>
+      <c r="Z6" s="3">
+        <v>1.0</v>
+      </c>
+      <c r="AA6" s="2" t="s">
+        <v>44</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="10">
+    <mergeCell ref="G5:H5"/>
+    <mergeCell ref="G6:H6"/>
+    <mergeCell ref="G2:H2"/>
+    <mergeCell ref="I2:J2"/>
+    <mergeCell ref="G3:H3"/>
+    <mergeCell ref="I3:J3"/>
+    <mergeCell ref="G4:H4"/>
+    <mergeCell ref="I4:J4"/>
+    <mergeCell ref="I5:J5"/>
+    <mergeCell ref="I6:J6"/>
+  </mergeCells>
   <drawing r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
test data fixes and loggers added to database and dao utility
</commit_message>
<xml_diff>
--- a/src/test/resources/testData/PhoenixTestData.xlsx
+++ b/src/test/resources/testData/PhoenixTestData.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="105" uniqueCount="51">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="115" uniqueCount="51">
   <si>
     <t>username</t>
   </si>
@@ -499,9 +499,7 @@
     <col customWidth="1" min="2" max="2" width="13.38"/>
     <col customWidth="1" min="3" max="3" width="19.0"/>
     <col customWidth="1" min="4" max="4" width="10.38"/>
-    <col customWidth="1" min="6" max="6" width="17.63"/>
-    <col customWidth="1" min="7" max="7" width="21.75"/>
-    <col customWidth="1" min="8" max="8" width="24.63"/>
+    <col customWidth="1" min="6" max="8" width="17.63"/>
     <col customWidth="1" min="19" max="19" width="21.13"/>
     <col customWidth="1" min="20" max="20" width="27.38"/>
     <col customWidth="1" min="21" max="22" width="20.75"/>
@@ -613,7 +611,13 @@
       <c r="G2" s="2" t="s">
         <v>34</v>
       </c>
+      <c r="H2" s="2" t="s">
+        <v>34</v>
+      </c>
       <c r="I2" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="J2" s="2" t="s">
         <v>35</v>
       </c>
       <c r="K2" s="2" t="s">
@@ -690,7 +694,13 @@
       <c r="G3" s="2" t="s">
         <v>34</v>
       </c>
+      <c r="H3" s="2" t="s">
+        <v>34</v>
+      </c>
       <c r="I3" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="J3" s="2" t="s">
         <v>35</v>
       </c>
       <c r="K3" s="2" t="s">
@@ -767,7 +777,13 @@
       <c r="G4" s="2" t="s">
         <v>34</v>
       </c>
+      <c r="H4" s="2" t="s">
+        <v>34</v>
+      </c>
       <c r="I4" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="J4" s="2" t="s">
         <v>35</v>
       </c>
       <c r="K4" s="2" t="s">
@@ -844,7 +860,13 @@
       <c r="G5" s="2" t="s">
         <v>34</v>
       </c>
+      <c r="H5" s="2" t="s">
+        <v>34</v>
+      </c>
       <c r="I5" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="J5" s="2" t="s">
         <v>35</v>
       </c>
       <c r="K5" s="2" t="s">
@@ -921,9 +943,15 @@
       <c r="G6" s="2" t="s">
         <v>34</v>
       </c>
+      <c r="H6" s="2" t="s">
+        <v>34</v>
+      </c>
       <c r="I6" s="2" t="s">
         <v>35</v>
       </c>
+      <c r="J6" s="2" t="s">
+        <v>35</v>
+      </c>
       <c r="K6" s="2" t="s">
         <v>36</v>
       </c>
@@ -977,18 +1005,6 @@
       </c>
     </row>
   </sheetData>
-  <mergeCells count="10">
-    <mergeCell ref="G5:H5"/>
-    <mergeCell ref="G6:H6"/>
-    <mergeCell ref="G2:H2"/>
-    <mergeCell ref="I2:J2"/>
-    <mergeCell ref="G3:H3"/>
-    <mergeCell ref="I3:J3"/>
-    <mergeCell ref="G4:H4"/>
-    <mergeCell ref="I4:J4"/>
-    <mergeCell ref="I5:J5"/>
-    <mergeCell ref="I6:J6"/>
-  </mergeCells>
   <drawing r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>